<commit_message>
Updated today at 10:02 PM 06-Sep
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>Felt tired after classes and had talked with new friends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile Screen time - 5h 20m </t>
   </si>
 </sst>
 </file>
@@ -1817,26 +1820,50 @@
       <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B24" s="14">
+        <v>420</v>
+      </c>
+      <c r="C24" s="14">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14">
+        <v>240</v>
+      </c>
+      <c r="E24" s="14">
+        <v>60</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>300</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:19 PM 07-Sep
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mobile Screen time - 5h 20m </t>
+  </si>
+  <si>
+    <t>Mobil screen time - 3h 52m</t>
   </si>
 </sst>
 </file>
@@ -1866,26 +1869,50 @@
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+      <c r="A25" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B25" s="14">
+        <v>390</v>
+      </c>
+      <c r="C25" s="14">
+        <v>120</v>
+      </c>
+      <c r="D25" s="14">
+        <v>180</v>
+      </c>
+      <c r="E25" s="14">
+        <v>0</v>
+      </c>
+      <c r="F25" s="14">
+        <v>200</v>
+      </c>
+      <c r="G25" s="14">
+        <v>4</v>
+      </c>
+      <c r="H25" s="14">
+        <v>180</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
+        <v>370</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="13"/>

</xml_diff>

<commit_message>
Updated today at 10:06 PM 08-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -243,6 +243,9 @@
   </si>
   <si>
     <t>Mobil screen time - 3h 52m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done with CA1 of DBMS (Mobile Screen time - 2h 12m </t>
   </si>
 </sst>
 </file>
@@ -1914,27 +1917,51 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+    <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B26" s="14">
+        <v>390</v>
+      </c>
+      <c r="C26" s="14">
+        <v>120</v>
+      </c>
+      <c r="D26" s="14">
+        <v>120</v>
+      </c>
+      <c r="E26" s="14">
+        <v>60</v>
+      </c>
+      <c r="F26" s="14">
+        <v>350</v>
+      </c>
+      <c r="G26" s="14">
+        <v>7</v>
+      </c>
+      <c r="H26" s="14">
+        <v>120</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
+        <v>280</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:56 PM 10-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t xml:space="preserve">Done with CA1 of DBMS (Mobile Screen time - 2h 12m </t>
+  </si>
+  <si>
+    <t>Today, I went to our freshers party after the classes  (mobile scrren time - 4h 20m )</t>
   </si>
 </sst>
 </file>
@@ -1963,27 +1966,51 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+    <row r="27" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B27" s="14">
+        <v>390</v>
+      </c>
+      <c r="C27" s="14">
+        <v>120</v>
+      </c>
+      <c r="D27" s="14">
+        <v>0</v>
+      </c>
+      <c r="E27" s="14">
+        <v>0</v>
+      </c>
+      <c r="F27" s="14">
+        <v>150</v>
+      </c>
+      <c r="G27" s="14">
+        <v>3</v>
+      </c>
+      <c r="H27" s="14">
+        <v>390</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:11 PM 11-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>Today, I went to our freshers party after the classes  (mobile scrren time - 4h 20m )</t>
+  </si>
+  <si>
+    <t>Today's mobile screen time is 3h 3 m</t>
   </si>
 </sst>
 </file>
@@ -2012,27 +2015,51 @@
         <v>70</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+    <row r="28" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B28" s="14">
+        <v>360</v>
+      </c>
+      <c r="C28" s="14">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14">
+        <v>240</v>
+      </c>
+      <c r="E28" s="14">
+        <v>180</v>
+      </c>
+      <c r="F28" s="14">
+        <v>250</v>
+      </c>
+      <c r="G28" s="14">
+        <v>5</v>
+      </c>
+      <c r="H28" s="14">
+        <v>300</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1330</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>110</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="13"/>

</xml_diff>

<commit_message>
Updated today at 12:39 PM 13-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="74">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -252,6 +252,12 @@
   </si>
   <si>
     <t>Today's mobile screen time is 3h 3 m</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>Had a great day today ! (mobile screen time 3h 20m</t>
   </si>
 </sst>
 </file>
@@ -2061,27 +2067,51 @@
         <v>71</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+    <row r="29" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B29" s="14">
+        <v>360</v>
+      </c>
+      <c r="C29" s="14">
+        <v>0</v>
+      </c>
+      <c r="D29" s="14">
+        <v>360</v>
+      </c>
+      <c r="E29" s="14">
+        <v>300</v>
+      </c>
+      <c r="F29" s="14">
+        <v>0</v>
+      </c>
+      <c r="G29" s="14">
+        <v>0</v>
+      </c>
+      <c r="H29" s="14">
+        <v>240</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1260</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
+        <v>180</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:50 PM 13-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t>Had a great day today ! (mobile screen time 3h 20m</t>
+  </si>
+  <si>
+    <t>I decided to change my full day schedule (Mobile Screen time - 1h 48m)</t>
   </si>
 </sst>
 </file>
@@ -2113,27 +2116,51 @@
         <v>73</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+    <row r="30" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B30" s="14">
+        <v>450</v>
+      </c>
+      <c r="C30" s="14">
+        <v>0</v>
+      </c>
+      <c r="D30" s="14">
+        <v>420</v>
+      </c>
+      <c r="E30" s="14">
+        <v>180</v>
+      </c>
+      <c r="F30" s="14">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14">
+        <v>360</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1410</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
+        <v>30</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:27 PM 14-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>I decided to change my full day schedule (Mobile Screen time - 1h 48m)</t>
+  </si>
+  <si>
+    <t>Got tired after the classes (Mobile screen time- 2h 43m</t>
   </si>
 </sst>
 </file>
@@ -2162,27 +2165,51 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+    <row r="31" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B31" s="14">
+        <v>420</v>
+      </c>
+      <c r="C31" s="14">
+        <v>120</v>
+      </c>
+      <c r="D31" s="14">
+        <v>90</v>
+      </c>
+      <c r="E31" s="14">
+        <v>90</v>
+      </c>
+      <c r="F31" s="14">
+        <v>200</v>
+      </c>
+      <c r="G31" s="14">
+        <v>3</v>
+      </c>
+      <c r="H31" s="14">
+        <v>390</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1310</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>130</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>

</xml_diff>

<commit_message>
Updated today at 1:35 PM 16-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -264,6 +264,9 @@
   </si>
   <si>
     <t>Got tired after the classes (Mobile screen time- 2h 43m</t>
+  </si>
+  <si>
+    <t>Explored MARS platform and gave CA and went out with friends</t>
   </si>
 </sst>
 </file>
@@ -2211,27 +2214,51 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+    <row r="32" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B32" s="14">
+        <v>360</v>
+      </c>
+      <c r="C32" s="14">
+        <v>120</v>
+      </c>
+      <c r="D32" s="14">
+        <v>0</v>
+      </c>
+      <c r="E32" s="14">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14">
+        <v>350</v>
+      </c>
+      <c r="G32" s="14">
+        <v>7</v>
+      </c>
+      <c r="H32" s="14">
+        <v>390</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
+        <v>220</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>

</xml_diff>

<commit_message>
Updated today at 12:54 AM 17-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -267,6 +267,9 @@
   </si>
   <si>
     <t>Explored MARS platform and gave CA and went out with friends</t>
+  </si>
+  <si>
+    <t>Tired after the classes</t>
   </si>
 </sst>
 </file>
@@ -2261,26 +2264,50 @@
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+      <c r="A33" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B33" s="14">
+        <v>480</v>
+      </c>
+      <c r="C33" s="14">
+        <v>120</v>
+      </c>
+      <c r="D33" s="14">
+        <v>150</v>
+      </c>
+      <c r="E33" s="14">
+        <v>0</v>
+      </c>
+      <c r="F33" s="14">
+        <v>350</v>
+      </c>
+      <c r="G33" s="14">
+        <v>7</v>
+      </c>
+      <c r="H33" s="14">
+        <v>300</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1400</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
+        <v>40</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:12 PM 17-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>Tired after the classes</t>
+  </si>
+  <si>
+    <t>Mobile screen time - 3h 30m</t>
   </si>
 </sst>
 </file>
@@ -2310,26 +2313,50 @@
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+      <c r="A34" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B34" s="14">
+        <v>510</v>
+      </c>
+      <c r="C34" s="14">
+        <v>120</v>
+      </c>
+      <c r="D34" s="14">
+        <v>300</v>
+      </c>
+      <c r="E34" s="14">
+        <v>0</v>
+      </c>
+      <c r="F34" s="14">
+        <v>200</v>
+      </c>
+      <c r="G34" s="14">
+        <v>4</v>
+      </c>
+      <c r="H34" s="14">
+        <v>300</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>1430</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
+        <v>10</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>

</xml_diff>

<commit_message>
Updated today at 12:29 AM 19-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -273,6 +273,9 @@
   </si>
   <si>
     <t>Mobile screen time - 3h 30m</t>
+  </si>
+  <si>
+    <t>Mobile screen time 4h 25m</t>
   </si>
 </sst>
 </file>
@@ -2359,26 +2362,50 @@
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+      <c r="A35" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B35" s="14">
+        <v>360</v>
+      </c>
+      <c r="C35" s="14">
+        <v>120</v>
+      </c>
+      <c r="D35" s="14">
+        <v>180</v>
+      </c>
+      <c r="E35" s="14">
+        <v>0</v>
+      </c>
+      <c r="F35" s="14">
+        <v>250</v>
+      </c>
+      <c r="G35" s="14">
+        <v>5</v>
+      </c>
+      <c r="H35" s="14">
+        <v>400</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1310</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
+        <v>130</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>

</xml_diff>

<commit_message>
Updated today at 12:20 AM 20-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -276,6 +276,9 @@
   </si>
   <si>
     <t>Mobile screen time 4h 25m</t>
+  </si>
+  <si>
+    <t>Used too much mobile today and got very sick</t>
   </si>
 </sst>
 </file>
@@ -2407,27 +2410,51 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+    <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="13">
+        <v>46284</v>
+      </c>
+      <c r="B36" s="14">
+        <v>360</v>
+      </c>
+      <c r="C36" s="14">
+        <v>120</v>
+      </c>
+      <c r="D36" s="14">
+        <v>120</v>
+      </c>
+      <c r="E36" s="14">
+        <v>60</v>
+      </c>
+      <c r="F36" s="14">
+        <v>0</v>
+      </c>
+      <c r="G36" s="14">
+        <v>0</v>
+      </c>
+      <c r="H36" s="14">
+        <v>600</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1260</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
+        <v>180</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:30 PM 23-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -279,6 +279,15 @@
   </si>
   <si>
     <t>Used too much mobile today and got very sick</t>
+  </si>
+  <si>
+    <t>Low energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">felt tired after the classes </t>
+  </si>
+  <si>
+    <t>felt tired after the classes (mobile screen time 2h 20m)</t>
   </si>
 </sst>
 </file>
@@ -2457,95 +2466,191 @@
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+      <c r="A37" s="13">
+        <v>46285</v>
+      </c>
+      <c r="B37" s="14">
+        <v>360</v>
+      </c>
+      <c r="C37" s="14">
+        <v>120</v>
+      </c>
+      <c r="D37" s="14">
+        <v>60</v>
+      </c>
+      <c r="E37" s="14">
+        <v>60</v>
+      </c>
+      <c r="F37" s="14">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14">
+        <v>0</v>
+      </c>
+      <c r="H37" s="14">
+        <v>600</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
+        <v>240</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+      <c r="A38" s="13">
+        <v>46286</v>
+      </c>
+      <c r="B38" s="14">
+        <v>360</v>
+      </c>
+      <c r="C38" s="14">
+        <v>120</v>
+      </c>
+      <c r="D38" s="14">
+        <v>180</v>
+      </c>
+      <c r="E38" s="14">
+        <v>0</v>
+      </c>
+      <c r="F38" s="14">
+        <v>200</v>
+      </c>
+      <c r="G38" s="14">
+        <v>4</v>
+      </c>
+      <c r="H38" s="14">
+        <v>500</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1360</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
+        <v>80</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N38" s="17"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+      <c r="A39" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B39" s="14">
+        <v>360</v>
+      </c>
+      <c r="C39" s="14">
+        <v>120</v>
+      </c>
+      <c r="D39" s="14">
+        <v>120</v>
+      </c>
+      <c r="E39" s="14">
+        <v>60</v>
+      </c>
+      <c r="F39" s="14">
+        <v>350</v>
+      </c>
+      <c r="G39" s="14">
+        <v>7</v>
+      </c>
+      <c r="H39" s="14">
+        <v>350</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1360</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+        <v>80</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="13">
+        <v>46288</v>
+      </c>
+      <c r="B40" s="14">
+        <v>360</v>
+      </c>
+      <c r="C40" s="14">
+        <v>120</v>
+      </c>
+      <c r="D40" s="14">
+        <v>180</v>
+      </c>
+      <c r="E40" s="14">
+        <v>150</v>
+      </c>
+      <c r="F40" s="14">
+        <v>350</v>
+      </c>
+      <c r="G40" s="14">
+        <v>6</v>
+      </c>
+      <c r="H40" s="14">
+        <v>280</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
+      <c r="A41" s="13">
+        <v>46289</v>
+      </c>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
       <c r="D41" s="14"/>
@@ -2567,7 +2672,9 @@
       <c r="N41" s="17"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
+      <c r="A42" s="13">
+        <v>46290</v>
+      </c>
       <c r="B42" s="14"/>
       <c r="C42" s="14"/>
       <c r="D42" s="14"/>
@@ -2589,7 +2696,9 @@
       <c r="N42" s="17"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
+      <c r="A43" s="13">
+        <v>46291</v>
+      </c>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
       <c r="D43" s="14"/>
@@ -2611,7 +2720,9 @@
       <c r="N43" s="17"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
+      <c r="A44" s="13">
+        <v>46292</v>
+      </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
@@ -2633,7 +2744,9 @@
       <c r="N44" s="17"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
+      <c r="A45" s="13">
+        <v>46293</v>
+      </c>
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
       <c r="D45" s="14"/>
@@ -2655,7 +2768,9 @@
       <c r="N45" s="17"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
+      <c r="A46" s="13">
+        <v>46294</v>
+      </c>
       <c r="B46" s="14"/>
       <c r="C46" s="14"/>
       <c r="D46" s="14"/>
@@ -2677,7 +2792,9 @@
       <c r="N46" s="17"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
+      <c r="A47" s="13">
+        <v>46295</v>
+      </c>
       <c r="B47" s="14"/>
       <c r="C47" s="14"/>
       <c r="D47" s="14"/>
@@ -2699,7 +2816,9 @@
       <c r="N47" s="17"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
+      <c r="A48" s="13">
+        <v>46296</v>
+      </c>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
       <c r="D48" s="14"/>

</xml_diff>

<commit_message>
Updated today at 10:51 PM 24-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="85">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -288,6 +288,9 @@
   </si>
   <si>
     <t>felt tired after the classes (mobile screen time 2h 20m)</t>
+  </si>
+  <si>
+    <t>Used too much mobile today..</t>
   </si>
 </sst>
 </file>
@@ -2651,25 +2654,47 @@
       <c r="A41" s="13">
         <v>46289</v>
       </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+      <c r="B41" s="14">
+        <v>420</v>
+      </c>
+      <c r="C41" s="14">
+        <v>120</v>
+      </c>
+      <c r="D41" s="14">
+        <v>60</v>
+      </c>
+      <c r="E41" s="14">
+        <v>60</v>
+      </c>
+      <c r="F41" s="14">
+        <v>200</v>
+      </c>
+      <c r="G41" s="14">
+        <v>4</v>
+      </c>
+      <c r="H41" s="14">
+        <v>400</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>1260</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
+        <v>180</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="13">

</xml_diff>

<commit_message>
Updated today at 12:24 AM 26-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -291,6 +291,9 @@
   </si>
   <si>
     <t>Used too much mobile today..</t>
+  </si>
+  <si>
+    <t>Had a great day today</t>
   </si>
 </sst>
 </file>
@@ -2700,25 +2703,47 @@
       <c r="A42" s="13">
         <v>46290</v>
       </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+      <c r="B42" s="14">
+        <v>420</v>
+      </c>
+      <c r="C42" s="14">
+        <v>120</v>
+      </c>
+      <c r="D42" s="14">
+        <v>120</v>
+      </c>
+      <c r="E42" s="14">
+        <v>120</v>
+      </c>
+      <c r="F42" s="14">
+        <v>250</v>
+      </c>
+      <c r="G42" s="14">
+        <v>5</v>
+      </c>
+      <c r="H42" s="14">
+        <v>400</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>1430</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
+        <v>10</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N42" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="13">

</xml_diff>

<commit_message>
Updated today at 4 PM 28-Sept
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -294,6 +294,15 @@
   </si>
   <si>
     <t>Had a great day today</t>
+  </si>
+  <si>
+    <t>Stressed</t>
+  </si>
+  <si>
+    <t>Very Unsatisfied</t>
+  </si>
+  <si>
+    <t>everything got changed all of sudden</t>
   </si>
 </sst>
 </file>
@@ -2749,49 +2758,91 @@
       <c r="A43" s="13">
         <v>46291</v>
       </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+      <c r="B43" s="14">
+        <v>420</v>
+      </c>
+      <c r="C43" s="14">
+        <v>0</v>
+      </c>
+      <c r="D43" s="14">
+        <v>120</v>
+      </c>
+      <c r="E43" s="14">
+        <v>120</v>
+      </c>
+      <c r="F43" s="14">
+        <v>0</v>
+      </c>
+      <c r="G43" s="14">
+        <v>0</v>
+      </c>
+      <c r="H43" s="14">
+        <v>700</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>1360</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
+        <v>80</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N43" s="17"/>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="13">
         <v>46292</v>
       </c>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+      <c r="B44" s="14">
+        <v>300</v>
+      </c>
+      <c r="C44" s="14">
+        <v>0</v>
+      </c>
+      <c r="D44" s="14">
+        <v>0</v>
+      </c>
+      <c r="E44" s="14">
+        <v>0</v>
+      </c>
+      <c r="F44" s="14">
+        <v>0</v>
+      </c>
+      <c r="G44" s="14">
+        <v>0</v>
+      </c>
+      <c r="H44" s="14">
+        <v>1100</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>1400</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="17"/>
+        <v>40</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="13">

</xml_diff>

<commit_message>
Updated today at 1:25 PM 04-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -300,9 +300,6 @@
   </si>
   <si>
     <t>Very Unsatisfied</t>
-  </si>
-  <si>
-    <t>everything got changed all of sudden</t>
   </si>
 </sst>
 </file>
@@ -2798,7 +2795,7 @@
       </c>
       <c r="N43" s="17"/>
     </row>
-    <row r="44" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="13">
         <v>46292</v>
       </c>
@@ -2840,166 +2837,292 @@
       <c r="M44" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="N44" s="17" t="s">
-        <v>88</v>
-      </c>
+      <c r="N44" s="17"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="13">
         <v>46293</v>
       </c>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+      <c r="B45" s="14">
+        <v>420</v>
+      </c>
+      <c r="C45" s="14">
+        <v>120</v>
+      </c>
+      <c r="D45" s="14">
+        <v>0</v>
+      </c>
+      <c r="E45" s="14">
+        <v>0</v>
+      </c>
+      <c r="F45" s="14">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14">
+        <v>0</v>
+      </c>
+      <c r="H45" s="14">
+        <v>900</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N45" s="17"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="13">
         <v>46294</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+      <c r="B46" s="14">
+        <v>420</v>
+      </c>
+      <c r="C46" s="14">
+        <v>120</v>
+      </c>
+      <c r="D46" s="14">
+        <v>0</v>
+      </c>
+      <c r="E46" s="14">
+        <v>0</v>
+      </c>
+      <c r="F46" s="14">
+        <v>0</v>
+      </c>
+      <c r="G46" s="14">
+        <v>0</v>
+      </c>
+      <c r="H46" s="14">
+        <v>900</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N46" s="17"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="13">
         <v>46295</v>
       </c>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
+      <c r="B47" s="14">
+        <v>360</v>
+      </c>
+      <c r="C47" s="14">
+        <v>120</v>
+      </c>
+      <c r="D47" s="14">
+        <v>180</v>
+      </c>
+      <c r="E47" s="14">
+        <v>120</v>
+      </c>
+      <c r="F47" s="14">
+        <v>0</v>
+      </c>
+      <c r="G47" s="14">
+        <v>0</v>
+      </c>
+      <c r="H47" s="14">
+        <v>660</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="N47" s="17"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="13">
         <v>46296</v>
       </c>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
+      <c r="B48" s="14">
+        <v>420</v>
+      </c>
+      <c r="C48" s="14">
+        <v>120</v>
+      </c>
+      <c r="D48" s="14">
+        <v>60</v>
+      </c>
+      <c r="E48" s="14">
+        <v>60</v>
+      </c>
+      <c r="F48" s="14">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14">
+        <v>780</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N48" s="17"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+      <c r="A49" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B49" s="14">
+        <v>420</v>
+      </c>
+      <c r="C49" s="14">
+        <v>0</v>
+      </c>
+      <c r="D49" s="14">
+        <v>0</v>
+      </c>
+      <c r="E49" s="14">
+        <v>0</v>
+      </c>
+      <c r="F49" s="14">
+        <v>0</v>
+      </c>
+      <c r="G49" s="14">
+        <v>0</v>
+      </c>
+      <c r="H49" s="14">
+        <v>1020</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N49" s="17"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+      <c r="A50" s="13">
+        <v>46298</v>
+      </c>
+      <c r="B50" s="14">
+        <v>480</v>
+      </c>
+      <c r="C50" s="14">
+        <v>120</v>
+      </c>
+      <c r="D50" s="14">
+        <v>120</v>
+      </c>
+      <c r="E50" s="14">
+        <v>0</v>
+      </c>
+      <c r="F50" s="14">
+        <v>0</v>
+      </c>
+      <c r="G50" s="14">
+        <v>0</v>
+      </c>
+      <c r="H50" s="14">
+        <v>720</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N50" s="17"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
+      <c r="A51" s="13">
+        <v>46299</v>
+      </c>
+      <c r="B51" s="14">
+        <v>480</v>
+      </c>
       <c r="C51" s="14"/>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
       <c r="F51" s="14"/>
       <c r="G51" s="14"/>
       <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>480</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
+        <v>960</v>
       </c>
       <c r="K51" s="16"/>
       <c r="L51" s="16"/>
@@ -3007,7 +3130,9 @@
       <c r="N51" s="17"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
+      <c r="A52" s="13">
+        <v>46300</v>
+      </c>
       <c r="B52" s="14"/>
       <c r="C52" s="14"/>
       <c r="D52" s="14"/>
@@ -3029,7 +3154,9 @@
       <c r="N52" s="17"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
+      <c r="A53" s="13">
+        <v>46301</v>
+      </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
       <c r="D53" s="14"/>
@@ -3051,7 +3178,9 @@
       <c r="N53" s="17"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="13"/>
+      <c r="A54" s="13">
+        <v>46302</v>
+      </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
       <c r="D54" s="14"/>
@@ -3073,7 +3202,9 @@
       <c r="N54" s="17"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="13"/>
+      <c r="A55" s="13">
+        <v>46303</v>
+      </c>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
       <c r="D55" s="14"/>
@@ -3095,7 +3226,9 @@
       <c r="N55" s="17"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="13"/>
+      <c r="A56" s="13">
+        <v>46304</v>
+      </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
       <c r="D56" s="14"/>
@@ -3117,7 +3250,9 @@
       <c r="N56" s="17"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="13"/>
+      <c r="A57" s="13">
+        <v>46305</v>
+      </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
       <c r="D57" s="14"/>

</xml_diff>

<commit_message>
Updated today at 10:45 PM 04-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3110,23 +3110,41 @@
       <c r="B51" s="14">
         <v>480</v>
       </c>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
+      <c r="C51" s="14">
+        <v>0</v>
+      </c>
+      <c r="D51" s="14">
+        <v>120</v>
+      </c>
+      <c r="E51" s="14">
+        <v>60</v>
+      </c>
+      <c r="F51" s="14">
+        <v>0</v>
+      </c>
+      <c r="G51" s="14">
+        <v>0</v>
+      </c>
+      <c r="H51" s="14">
+        <v>780</v>
+      </c>
       <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v>480</v>
+        <v>1440</v>
       </c>
       <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v>960</v>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N51" s="17"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 10:40 PM 05-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>Very Unsatisfied</t>
+  </si>
+  <si>
+    <t>feeling sick</t>
   </si>
 </sst>
 </file>
@@ -3151,25 +3154,47 @@
       <c r="A52" s="13">
         <v>46300</v>
       </c>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+      <c r="B52" s="14">
+        <v>420</v>
+      </c>
+      <c r="C52" s="14">
+        <v>60</v>
+      </c>
+      <c r="D52" s="14">
+        <v>120</v>
+      </c>
+      <c r="E52" s="14">
+        <v>0</v>
+      </c>
+      <c r="F52" s="14">
+        <v>200</v>
+      </c>
+      <c r="G52" s="14">
+        <v>4</v>
+      </c>
+      <c r="H52" s="14">
+        <v>640</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="13">

</xml_diff>

<commit_message>
Updated today at 10:33 PM 06-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -303,6 +303,9 @@
   </si>
   <si>
     <t>feeling sick</t>
+  </si>
+  <si>
+    <t>Less screen time, more focused on study and talked with strangers in english</t>
   </si>
 </sst>
 </file>
@@ -3196,29 +3199,51 @@
         <v>88</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A53" s="13">
         <v>46301</v>
       </c>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+      <c r="B53" s="14">
+        <v>420</v>
+      </c>
+      <c r="C53" s="14">
+        <v>90</v>
+      </c>
+      <c r="D53" s="14">
+        <v>180</v>
+      </c>
+      <c r="E53" s="14">
+        <v>0</v>
+      </c>
+      <c r="F53" s="14">
+        <v>350</v>
+      </c>
+      <c r="G53" s="14">
+        <v>7</v>
+      </c>
+      <c r="H53" s="14">
+        <v>400</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="17"/>
+        <v>0</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N53" s="17" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="13">

</xml_diff>

<commit_message>
Updated today at 11:13 PM 07-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3249,24 +3249,44 @@
       <c r="A54" s="13">
         <v>46302</v>
       </c>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="15" t="str">
+      <c r="B54" s="14">
+        <v>360</v>
+      </c>
+      <c r="C54" s="14">
+        <v>90</v>
+      </c>
+      <c r="D54" s="14">
+        <v>120</v>
+      </c>
+      <c r="E54" s="14">
+        <v>0</v>
+      </c>
+      <c r="F54" s="14">
+        <v>350</v>
+      </c>
+      <c r="G54" s="14">
+        <v>7</v>
+      </c>
+      <c r="H54" s="14">
+        <v>520</v>
+      </c>
+      <c r="I54" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J54" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="16"/>
-      <c r="M54" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K54" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L54" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M54" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N54" s="17"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 11:07 PM 08-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3293,24 +3293,44 @@
       <c r="A55" s="13">
         <v>46303</v>
       </c>
-      <c r="B55" s="14"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="15" t="str">
+      <c r="B55" s="14">
+        <v>360</v>
+      </c>
+      <c r="C55" s="14">
+        <v>90</v>
+      </c>
+      <c r="D55" s="14">
+        <v>120</v>
+      </c>
+      <c r="E55" s="14">
+        <v>0</v>
+      </c>
+      <c r="F55" s="14">
+        <v>0</v>
+      </c>
+      <c r="G55" s="14">
+        <v>0</v>
+      </c>
+      <c r="H55" s="14">
+        <v>870</v>
+      </c>
+      <c r="I55" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J55" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="16"/>
-      <c r="L55" s="16"/>
-      <c r="M55" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K55" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L55" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M55" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N55" s="17"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 10:35 PM 10-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3337,52 +3337,94 @@
       <c r="A56" s="13">
         <v>46304</v>
       </c>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="14"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="15" t="str">
+      <c r="B56" s="14">
+        <v>420</v>
+      </c>
+      <c r="C56" s="14">
+        <v>0</v>
+      </c>
+      <c r="D56" s="14">
+        <v>180</v>
+      </c>
+      <c r="E56" s="14">
+        <v>0</v>
+      </c>
+      <c r="F56" s="14">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14">
+        <v>840</v>
+      </c>
+      <c r="I56" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J56" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="16"/>
-      <c r="M56" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L56" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M56" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N56" s="17"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="13">
         <v>46305</v>
       </c>
-      <c r="B57" s="14"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="14"/>
-      <c r="H57" s="14"/>
-      <c r="I57" s="15" t="str">
+      <c r="B57" s="14">
+        <v>480</v>
+      </c>
+      <c r="C57" s="14">
+        <v>0</v>
+      </c>
+      <c r="D57" s="14">
+        <v>240</v>
+      </c>
+      <c r="E57" s="14">
+        <v>0</v>
+      </c>
+      <c r="F57" s="14">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14">
+        <v>0</v>
+      </c>
+      <c r="H57" s="14">
+        <v>720</v>
+      </c>
+      <c r="I57" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J57" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="16"/>
-      <c r="L57" s="16"/>
-      <c r="M57" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L57" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M57" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N57" s="17"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="13"/>
+      <c r="A58" s="13">
+        <v>46306</v>
+      </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
       <c r="D58" s="14"/>
@@ -3404,7 +3446,9 @@
       <c r="N58" s="17"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="13"/>
+      <c r="A59" s="13">
+        <v>46307</v>
+      </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
       <c r="D59" s="14"/>
@@ -3426,7 +3470,9 @@
       <c r="N59" s="17"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="13"/>
+      <c r="A60" s="13">
+        <v>46308</v>
+      </c>
       <c r="B60" s="14"/>
       <c r="C60" s="14"/>
       <c r="D60" s="14"/>
@@ -3448,7 +3494,9 @@
       <c r="N60" s="17"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="13"/>
+      <c r="A61" s="13">
+        <v>46309</v>
+      </c>
       <c r="B61" s="14"/>
       <c r="C61" s="14"/>
       <c r="D61" s="14"/>
@@ -3470,7 +3518,9 @@
       <c r="N61" s="17"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="13"/>
+      <c r="A62" s="13">
+        <v>46310</v>
+      </c>
       <c r="B62" s="14"/>
       <c r="C62" s="14"/>
       <c r="D62" s="14"/>
@@ -3492,7 +3542,9 @@
       <c r="N62" s="17"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="13"/>
+      <c r="A63" s="13">
+        <v>46311</v>
+      </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
@@ -3514,7 +3566,9 @@
       <c r="N63" s="17"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="13"/>
+      <c r="A64" s="13">
+        <v>46312</v>
+      </c>
       <c r="B64" s="14"/>
       <c r="C64" s="14"/>
       <c r="D64" s="14"/>
@@ -3536,7 +3590,9 @@
       <c r="N64" s="17"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A65" s="13"/>
+      <c r="A65" s="13">
+        <v>46313</v>
+      </c>
       <c r="B65" s="14"/>
       <c r="C65" s="14"/>
       <c r="D65" s="14"/>
@@ -3558,7 +3614,9 @@
       <c r="N65" s="17"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A66" s="13"/>
+      <c r="A66" s="13">
+        <v>46314</v>
+      </c>
       <c r="B66" s="14"/>
       <c r="C66" s="14"/>
       <c r="D66" s="14"/>
@@ -3580,7 +3638,9 @@
       <c r="N66" s="17"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A67" s="13"/>
+      <c r="A67" s="13">
+        <v>46315</v>
+      </c>
       <c r="B67" s="14"/>
       <c r="C67" s="14"/>
       <c r="D67" s="14"/>
@@ -3602,7 +3662,9 @@
       <c r="N67" s="17"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A68" s="13"/>
+      <c r="A68" s="13">
+        <v>46316</v>
+      </c>
       <c r="B68" s="14"/>
       <c r="C68" s="14"/>
       <c r="D68" s="14"/>
@@ -3624,7 +3686,9 @@
       <c r="N68" s="17"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="13"/>
+      <c r="A69" s="13">
+        <v>46317</v>
+      </c>
       <c r="B69" s="14"/>
       <c r="C69" s="14"/>
       <c r="D69" s="14"/>
@@ -3646,7 +3710,9 @@
       <c r="N69" s="17"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="13"/>
+      <c r="A70" s="13">
+        <v>46318</v>
+      </c>
       <c r="B70" s="14"/>
       <c r="C70" s="14"/>
       <c r="D70" s="14"/>

</xml_diff>

<commit_message>
Updated today at 10:12 PM 11-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3425,24 +3425,44 @@
       <c r="A58" s="13">
         <v>46306</v>
       </c>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="15" t="str">
+      <c r="B58" s="14">
+        <v>480</v>
+      </c>
+      <c r="C58" s="14">
+        <v>0</v>
+      </c>
+      <c r="D58" s="14">
+        <v>180</v>
+      </c>
+      <c r="E58" s="14">
+        <v>0</v>
+      </c>
+      <c r="F58" s="14">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14">
+        <v>0</v>
+      </c>
+      <c r="H58" s="14">
+        <v>780</v>
+      </c>
+      <c r="I58" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J58" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="16"/>
-      <c r="M58" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L58" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M58" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N58" s="17"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 12:04 AM 13-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3469,24 +3469,44 @@
       <c r="A59" s="13">
         <v>46307</v>
       </c>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="14"/>
-      <c r="H59" s="14"/>
-      <c r="I59" s="15" t="str">
+      <c r="B59" s="14">
+        <v>420</v>
+      </c>
+      <c r="C59" s="14">
+        <v>90</v>
+      </c>
+      <c r="D59" s="14">
+        <v>240</v>
+      </c>
+      <c r="E59" s="14">
+        <v>180</v>
+      </c>
+      <c r="F59" s="14">
+        <v>0</v>
+      </c>
+      <c r="G59" s="14">
+        <v>0</v>
+      </c>
+      <c r="H59" s="14">
+        <v>510</v>
+      </c>
+      <c r="I59" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J59" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="16"/>
-      <c r="L59" s="16"/>
-      <c r="M59" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L59" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M59" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N59" s="17"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 10:40 PM 14-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3513,48 +3513,88 @@
       <c r="A60" s="13">
         <v>46308</v>
       </c>
-      <c r="B60" s="14"/>
-      <c r="C60" s="14"/>
-      <c r="D60" s="14"/>
-      <c r="E60" s="14"/>
-      <c r="F60" s="14"/>
-      <c r="G60" s="14"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="15" t="str">
+      <c r="B60" s="14">
+        <v>420</v>
+      </c>
+      <c r="C60" s="14">
+        <v>90</v>
+      </c>
+      <c r="D60" s="14">
+        <v>240</v>
+      </c>
+      <c r="E60" s="14">
+        <v>0</v>
+      </c>
+      <c r="F60" s="14">
+        <v>0</v>
+      </c>
+      <c r="G60" s="14">
+        <v>0</v>
+      </c>
+      <c r="H60" s="14">
+        <v>690</v>
+      </c>
+      <c r="I60" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J60" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L60" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M60" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N60" s="17"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="13">
         <v>46309</v>
       </c>
-      <c r="B61" s="14"/>
-      <c r="C61" s="14"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="14"/>
-      <c r="I61" s="15" t="str">
+      <c r="B61" s="14">
+        <v>480</v>
+      </c>
+      <c r="C61" s="14">
+        <v>0</v>
+      </c>
+      <c r="D61" s="14">
+        <v>60</v>
+      </c>
+      <c r="E61" s="14">
+        <v>0</v>
+      </c>
+      <c r="F61" s="14">
+        <v>0</v>
+      </c>
+      <c r="G61" s="14">
+        <v>0</v>
+      </c>
+      <c r="H61" s="14">
+        <v>900</v>
+      </c>
+      <c r="I61" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J61" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K61" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L61" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M61" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N61" s="17"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 10:42 PM 21-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -492,7 +492,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1113,7 +1124,7 @@
         <v>885</v>
       </c>
       <c r="J6" s="10">
-        <f t="shared" ref="J6:J69" si="1">IF(I6="","",1440-I6)</f>
+        <f t="shared" ref="H6:J69" si="1">IF(I6="","",1440-I6)</f>
         <v>555</v>
       </c>
       <c r="K6" s="11" t="s">
@@ -3564,7 +3575,7 @@
         <v>0</v>
       </c>
       <c r="D61" s="14">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="E61" s="14">
         <v>0</v>
@@ -3576,7 +3587,7 @@
         <v>0</v>
       </c>
       <c r="H61" s="14">
-        <v>900</v>
+        <v>780</v>
       </c>
       <c r="I61" s="15">
         <f t="shared" si="0"/>
@@ -3601,168 +3612,308 @@
       <c r="A62" s="13">
         <v>46310</v>
       </c>
-      <c r="B62" s="14"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="15" t="str">
+      <c r="B62" s="14">
+        <v>480</v>
+      </c>
+      <c r="C62" s="14">
+        <v>0</v>
+      </c>
+      <c r="D62" s="14">
+        <v>120</v>
+      </c>
+      <c r="E62" s="14">
+        <v>0</v>
+      </c>
+      <c r="F62" s="14">
+        <v>0</v>
+      </c>
+      <c r="G62" s="14">
+        <v>0</v>
+      </c>
+      <c r="H62" s="14">
+        <v>840</v>
+      </c>
+      <c r="I62" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J62" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K62" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L62" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N62" s="17"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="13">
         <v>46311</v>
       </c>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="15" t="str">
+      <c r="B63" s="14">
+        <v>480</v>
+      </c>
+      <c r="C63" s="14">
+        <v>0</v>
+      </c>
+      <c r="D63" s="14">
+        <v>350</v>
+      </c>
+      <c r="E63" s="14">
+        <v>0</v>
+      </c>
+      <c r="F63" s="14">
+        <v>0</v>
+      </c>
+      <c r="G63" s="14">
+        <v>0</v>
+      </c>
+      <c r="H63" s="14">
+        <v>610</v>
+      </c>
+      <c r="I63" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J63" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="16"/>
-      <c r="L63" s="16"/>
-      <c r="M63" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K63" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L63" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N63" s="17"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="13">
         <v>46312</v>
       </c>
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="15" t="str">
+      <c r="B64" s="14">
+        <v>480</v>
+      </c>
+      <c r="C64" s="14">
+        <v>0</v>
+      </c>
+      <c r="D64" s="14">
+        <v>240</v>
+      </c>
+      <c r="E64" s="14">
+        <v>0</v>
+      </c>
+      <c r="F64" s="14">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14">
+        <v>0</v>
+      </c>
+      <c r="H64" s="14">
+        <v>720</v>
+      </c>
+      <c r="I64" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J64" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K64" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L64" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M64" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N64" s="17"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="13">
         <v>46313</v>
       </c>
-      <c r="B65" s="14"/>
-      <c r="C65" s="14"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="G65" s="14"/>
-      <c r="H65" s="14"/>
-      <c r="I65" s="15" t="str">
+      <c r="B65" s="14">
+        <v>480</v>
+      </c>
+      <c r="C65" s="14">
+        <v>0</v>
+      </c>
+      <c r="D65" s="14">
+        <v>120</v>
+      </c>
+      <c r="E65" s="14">
+        <v>0</v>
+      </c>
+      <c r="F65" s="14">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14">
+        <v>0</v>
+      </c>
+      <c r="H65" s="14">
+        <v>840</v>
+      </c>
+      <c r="I65" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J65" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K65" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L65" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M65" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N65" s="17"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="13">
         <v>46314</v>
       </c>
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
-      <c r="F66" s="14"/>
-      <c r="G66" s="14"/>
-      <c r="H66" s="14"/>
-      <c r="I66" s="15" t="str">
+      <c r="B66" s="14">
+        <v>480</v>
+      </c>
+      <c r="C66" s="14">
+        <v>0</v>
+      </c>
+      <c r="D66" s="14">
+        <v>120</v>
+      </c>
+      <c r="E66" s="14">
+        <v>0</v>
+      </c>
+      <c r="F66" s="14">
+        <v>200</v>
+      </c>
+      <c r="G66" s="14">
+        <v>4</v>
+      </c>
+      <c r="H66" s="14">
+        <v>640</v>
+      </c>
+      <c r="I66" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J66" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K66" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L66" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M66" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N66" s="17"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="13">
         <v>46315</v>
       </c>
-      <c r="B67" s="14"/>
-      <c r="C67" s="14"/>
-      <c r="D67" s="14"/>
-      <c r="E67" s="14"/>
-      <c r="F67" s="14"/>
-      <c r="G67" s="14"/>
-      <c r="H67" s="14"/>
-      <c r="I67" s="15" t="str">
+      <c r="B67" s="14">
+        <v>480</v>
+      </c>
+      <c r="C67" s="14">
+        <v>0</v>
+      </c>
+      <c r="D67" s="14">
+        <v>120</v>
+      </c>
+      <c r="E67" s="14">
+        <v>60</v>
+      </c>
+      <c r="F67" s="14">
+        <v>0</v>
+      </c>
+      <c r="G67" s="14">
+        <v>0</v>
+      </c>
+      <c r="H67" s="14">
+        <v>780</v>
+      </c>
+      <c r="I67" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J67" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J67" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K67" s="16"/>
-      <c r="L67" s="16"/>
-      <c r="M67" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K67" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L67" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M67" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="N67" s="17"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="13">
         <v>46316</v>
       </c>
-      <c r="B68" s="14"/>
-      <c r="C68" s="14"/>
-      <c r="D68" s="14"/>
-      <c r="E68" s="14"/>
-      <c r="F68" s="14"/>
-      <c r="G68" s="14"/>
-      <c r="H68" s="14"/>
-      <c r="I68" s="15" t="str">
+      <c r="B68" s="14">
+        <v>480</v>
+      </c>
+      <c r="C68" s="14">
+        <v>0</v>
+      </c>
+      <c r="D68" s="14">
+        <v>60</v>
+      </c>
+      <c r="E68" s="14">
+        <v>0</v>
+      </c>
+      <c r="F68" s="14">
+        <v>350</v>
+      </c>
+      <c r="G68" s="14">
+        <v>7</v>
+      </c>
+      <c r="H68" s="14">
+        <v>550</v>
+      </c>
+      <c r="I68" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J68" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K68" s="16"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K68" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L68" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M68" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N68" s="17"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
@@ -11105,7 +11256,7 @@
     <mergeCell ref="F3:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="J6:J401">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Updated today at 10:50 PM 22-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -492,18 +492,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1124,7 +1113,7 @@
         <v>885</v>
       </c>
       <c r="J6" s="10">
-        <f t="shared" ref="H6:J69" si="1">IF(I6="","",1440-I6)</f>
+        <f t="shared" ref="J6:J69" si="1">IF(I6="","",1440-I6)</f>
         <v>555</v>
       </c>
       <c r="K6" s="11" t="s">
@@ -3920,24 +3909,44 @@
       <c r="A69" s="13">
         <v>46317</v>
       </c>
-      <c r="B69" s="14"/>
-      <c r="C69" s="14"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14"/>
-      <c r="F69" s="14"/>
-      <c r="G69" s="14"/>
-      <c r="H69" s="14"/>
-      <c r="I69" s="15" t="str">
+      <c r="B69" s="14">
+        <v>420</v>
+      </c>
+      <c r="C69" s="14">
+        <v>60</v>
+      </c>
+      <c r="D69" s="14">
+        <v>60</v>
+      </c>
+      <c r="E69" s="14">
+        <v>0</v>
+      </c>
+      <c r="F69" s="14">
+        <v>200</v>
+      </c>
+      <c r="G69" s="14">
+        <v>3</v>
+      </c>
+      <c r="H69" s="14">
+        <v>700</v>
+      </c>
+      <c r="I69" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J69" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J69" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K69" s="16"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K69" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L69" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M69" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N69" s="17"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
@@ -11256,7 +11265,7 @@
     <mergeCell ref="F3:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="J6:J401">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Updated today at 11:16 PM 26-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3953,94 +3953,182 @@
       <c r="A70" s="13">
         <v>46318</v>
       </c>
-      <c r="B70" s="14"/>
-      <c r="C70" s="14"/>
-      <c r="D70" s="14"/>
-      <c r="E70" s="14"/>
-      <c r="F70" s="14"/>
-      <c r="G70" s="14"/>
-      <c r="H70" s="14"/>
-      <c r="I70" s="15" t="str">
+      <c r="B70" s="14">
+        <v>400</v>
+      </c>
+      <c r="C70" s="14">
+        <v>60</v>
+      </c>
+      <c r="D70" s="14">
+        <v>60</v>
+      </c>
+      <c r="E70" s="14">
+        <v>0</v>
+      </c>
+      <c r="F70" s="14">
+        <v>250</v>
+      </c>
+      <c r="G70" s="14">
+        <v>5</v>
+      </c>
+      <c r="H70" s="14">
+        <v>670</v>
+      </c>
+      <c r="I70" s="15">
         <f t="shared" ref="I70:I133" si="2">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
-        <v/>
-      </c>
-      <c r="J70" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J70" s="15">
         <f t="shared" ref="J70:J133" si="3">IF(I70="","",1440-I70)</f>
-        <v/>
-      </c>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K70" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L70" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M70" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N70" s="17"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="13"/>
-      <c r="B71" s="14"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
-      <c r="G71" s="14"/>
-      <c r="H71" s="14"/>
-      <c r="I71" s="15" t="str">
+      <c r="A71" s="13">
+        <v>46319</v>
+      </c>
+      <c r="B71" s="14">
+        <v>30</v>
+      </c>
+      <c r="C71" s="14">
+        <v>0</v>
+      </c>
+      <c r="D71" s="14">
+        <v>0</v>
+      </c>
+      <c r="E71" s="14">
+        <v>0</v>
+      </c>
+      <c r="F71" s="14">
+        <v>0</v>
+      </c>
+      <c r="G71" s="14">
+        <v>0</v>
+      </c>
+      <c r="H71" s="14">
+        <v>1410</v>
+      </c>
+      <c r="I71" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J71" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J71" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K71" s="16"/>
-      <c r="L71" s="16"/>
-      <c r="M71" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K71" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L71" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M71" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="N71" s="17"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="13"/>
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="15" t="str">
+      <c r="A72" s="13">
+        <v>46320</v>
+      </c>
+      <c r="B72" s="14">
+        <v>360</v>
+      </c>
+      <c r="C72" s="14">
+        <v>0</v>
+      </c>
+      <c r="D72" s="14">
+        <v>0</v>
+      </c>
+      <c r="E72" s="14">
+        <v>0</v>
+      </c>
+      <c r="F72" s="14">
+        <v>0</v>
+      </c>
+      <c r="G72" s="14">
+        <v>0</v>
+      </c>
+      <c r="H72" s="14">
+        <v>1080</v>
+      </c>
+      <c r="I72" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J72" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J72" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K72" s="16"/>
-      <c r="L72" s="16"/>
-      <c r="M72" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K72" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L72" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M72" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="N72" s="17"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A73" s="13"/>
-      <c r="B73" s="14"/>
-      <c r="C73" s="14"/>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
-      <c r="F73" s="14"/>
-      <c r="G73" s="14"/>
-      <c r="H73" s="14"/>
-      <c r="I73" s="15" t="str">
+      <c r="A73" s="13">
+        <v>46321</v>
+      </c>
+      <c r="B73" s="14">
+        <v>600</v>
+      </c>
+      <c r="C73" s="14">
+        <v>0</v>
+      </c>
+      <c r="D73" s="14">
+        <v>180</v>
+      </c>
+      <c r="E73" s="14">
+        <v>60</v>
+      </c>
+      <c r="F73" s="14">
+        <v>0</v>
+      </c>
+      <c r="G73" s="14">
+        <v>0</v>
+      </c>
+      <c r="H73" s="14">
+        <v>600</v>
+      </c>
+      <c r="I73" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J73" s="15" t="str">
+        <v>1440</v>
+      </c>
+      <c r="J73" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K73" s="16"/>
-      <c r="L73" s="16"/>
-      <c r="M73" s="16"/>
+        <v>0</v>
+      </c>
+      <c r="K73" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L73" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M73" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N73" s="17"/>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A74" s="13"/>
+      <c r="A74" s="13">
+        <v>46322</v>
+      </c>
       <c r="B74" s="14"/>
       <c r="C74" s="14"/>
       <c r="D74" s="14"/>
@@ -4062,7 +4150,9 @@
       <c r="N74" s="17"/>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A75" s="13"/>
+      <c r="A75" s="13">
+        <v>46323</v>
+      </c>
       <c r="B75" s="14"/>
       <c r="C75" s="14"/>
       <c r="D75" s="14"/>

</xml_diff>

<commit_message>
Updated today at 10:37 PM 27-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4129,24 +4129,44 @@
       <c r="A74" s="13">
         <v>46322</v>
       </c>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="14"/>
-      <c r="H74" s="14"/>
-      <c r="I74" s="15" t="str">
+      <c r="B74" s="14">
+        <v>480</v>
+      </c>
+      <c r="C74" s="14">
+        <v>0</v>
+      </c>
+      <c r="D74" s="14">
+        <v>120</v>
+      </c>
+      <c r="E74" s="14">
+        <v>120</v>
+      </c>
+      <c r="F74" s="14">
+        <v>200</v>
+      </c>
+      <c r="G74" s="14">
+        <v>4</v>
+      </c>
+      <c r="H74" s="14">
+        <v>360</v>
+      </c>
+      <c r="I74" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J74" s="15" t="str">
+        <v>1280</v>
+      </c>
+      <c r="J74" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K74" s="16"/>
-      <c r="L74" s="16"/>
-      <c r="M74" s="16"/>
+        <v>160</v>
+      </c>
+      <c r="K74" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L74" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M74" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N74" s="17"/>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 12:00 PM 31-oct
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4173,72 +4173,138 @@
       <c r="A75" s="13">
         <v>46323</v>
       </c>
-      <c r="B75" s="14"/>
-      <c r="C75" s="14"/>
-      <c r="D75" s="14"/>
-      <c r="E75" s="14"/>
-      <c r="F75" s="14"/>
-      <c r="G75" s="14"/>
-      <c r="H75" s="14"/>
-      <c r="I75" s="15" t="str">
+      <c r="B75" s="14">
+        <v>480</v>
+      </c>
+      <c r="C75" s="14">
+        <v>60</v>
+      </c>
+      <c r="D75" s="14">
+        <v>0</v>
+      </c>
+      <c r="E75" s="14">
+        <v>0</v>
+      </c>
+      <c r="F75" s="14">
+        <v>350</v>
+      </c>
+      <c r="G75" s="14">
+        <v>7</v>
+      </c>
+      <c r="H75" s="14">
+        <v>360</v>
+      </c>
+      <c r="I75" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J75" s="15" t="str">
+        <v>1250</v>
+      </c>
+      <c r="J75" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K75" s="16"/>
-      <c r="L75" s="16"/>
-      <c r="M75" s="16"/>
+        <v>190</v>
+      </c>
+      <c r="K75" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L75" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M75" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N75" s="17"/>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A76" s="13"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="14"/>
-      <c r="H76" s="14"/>
-      <c r="I76" s="15" t="str">
+      <c r="A76" s="13">
+        <v>46324</v>
+      </c>
+      <c r="B76" s="14">
+        <v>480</v>
+      </c>
+      <c r="C76" s="14">
+        <v>60</v>
+      </c>
+      <c r="D76" s="14">
+        <v>60</v>
+      </c>
+      <c r="E76" s="14">
+        <v>60</v>
+      </c>
+      <c r="F76" s="14">
+        <v>250</v>
+      </c>
+      <c r="G76" s="14">
+        <v>5</v>
+      </c>
+      <c r="H76" s="14">
+        <v>260</v>
+      </c>
+      <c r="I76" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J76" s="15" t="str">
+        <v>1170</v>
+      </c>
+      <c r="J76" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K76" s="16"/>
-      <c r="L76" s="16"/>
-      <c r="M76" s="16"/>
+        <v>270</v>
+      </c>
+      <c r="K76" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L76" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M76" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N76" s="17"/>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A77" s="13"/>
-      <c r="B77" s="14"/>
-      <c r="C77" s="14"/>
-      <c r="D77" s="14"/>
-      <c r="E77" s="14"/>
-      <c r="F77" s="14"/>
-      <c r="G77" s="14"/>
-      <c r="H77" s="14"/>
-      <c r="I77" s="15" t="str">
+      <c r="A77" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B77" s="14">
+        <v>360</v>
+      </c>
+      <c r="C77" s="14">
+        <v>120</v>
+      </c>
+      <c r="D77" s="14">
+        <v>120</v>
+      </c>
+      <c r="E77" s="14">
+        <v>60</v>
+      </c>
+      <c r="F77" s="14">
+        <v>250</v>
+      </c>
+      <c r="G77" s="14">
+        <v>5</v>
+      </c>
+      <c r="H77" s="14">
+        <v>350</v>
+      </c>
+      <c r="I77" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J77" s="15" t="str">
+        <v>1260</v>
+      </c>
+      <c r="J77" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K77" s="16"/>
-      <c r="L77" s="16"/>
-      <c r="M77" s="16"/>
+        <v>180</v>
+      </c>
+      <c r="K77" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L77" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M77" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N77" s="17"/>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A78" s="13"/>
+      <c r="A78" s="13">
+        <v>46326</v>
+      </c>
       <c r="B78" s="14"/>
       <c r="C78" s="14"/>
       <c r="D78" s="14"/>
@@ -4260,7 +4326,9 @@
       <c r="N78" s="17"/>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A79" s="13"/>
+      <c r="A79" s="13">
+        <v>46327</v>
+      </c>
       <c r="B79" s="14"/>
       <c r="C79" s="14"/>
       <c r="D79" s="14"/>
@@ -4282,7 +4350,9 @@
       <c r="N79" s="17"/>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A80" s="13"/>
+      <c r="A80" s="13">
+        <v>46328</v>
+      </c>
       <c r="B80" s="14"/>
       <c r="C80" s="14"/>
       <c r="D80" s="14"/>
@@ -4304,7 +4374,9 @@
       <c r="N80" s="17"/>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A81" s="13"/>
+      <c r="A81" s="13">
+        <v>46329</v>
+      </c>
       <c r="B81" s="14"/>
       <c r="C81" s="14"/>
       <c r="D81" s="14"/>
@@ -4326,7 +4398,9 @@
       <c r="N81" s="17"/>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A82" s="13"/>
+      <c r="A82" s="13">
+        <v>46330</v>
+      </c>
       <c r="B82" s="14"/>
       <c r="C82" s="14"/>
       <c r="D82" s="14"/>
@@ -4348,7 +4422,9 @@
       <c r="N82" s="17"/>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A83" s="13"/>
+      <c r="A83" s="13">
+        <v>46331</v>
+      </c>
       <c r="B83" s="14"/>
       <c r="C83" s="14"/>
       <c r="D83" s="14"/>
@@ -4370,7 +4446,9 @@
       <c r="N83" s="17"/>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A84" s="13"/>
+      <c r="A84" s="13">
+        <v>46332</v>
+      </c>
       <c r="B84" s="14"/>
       <c r="C84" s="14"/>
       <c r="D84" s="14"/>
@@ -4392,7 +4470,9 @@
       <c r="N84" s="17"/>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A85" s="13"/>
+      <c r="A85" s="13">
+        <v>46333</v>
+      </c>
       <c r="B85" s="14"/>
       <c r="C85" s="14"/>
       <c r="D85" s="14"/>

</xml_diff>